<commit_message>
Replace PSIN/OSL free-text codes with SDC openLabel and drop Mapping tab.
Use a single open-choice free-text label per question, remove the Additional Language code system, add the SDC dependency, and republish docs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-AHIP-Demo-Additional-NullFlavor.xlsx
+++ b/docs/CodeSystem-AHIP-Demo-Additional-NullFlavor.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="48">
   <si>
     <t>Property</t>
   </si>
@@ -123,7 +123,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>3</t>
+    <t>2</t>
   </si>
   <si>
     <t>Level</t>
@@ -157,15 +157,6 @@
   </si>
   <si>
     <t>**Description:**This code is to represent explicitly that the patient do not want a pronoun to be used but instead use their name</t>
-  </si>
-  <si>
-    <t>PSIN</t>
-  </si>
-  <si>
-    <t>Please specify if not listed above</t>
-  </si>
-  <si>
-    <t>**Description:**This code is to represent explicitly that the patient would like to specify a value that is not listed above</t>
   </si>
 </sst>
 </file>
@@ -475,7 +466,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -520,20 +511,6 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="B4" t="s" s="2">
-        <v>48</v>
-      </c>
-      <c r="C4" t="s" s="2">
-        <v>49</v>
-      </c>
-      <c r="D4" t="s" s="2">
-        <v>50</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>